<commit_message>
Solo gramos/mililitros/unidad en inventario y avisos de exito/error
Migra el catalogo de unidades de kg/l a solo g/ml/unidad (con reescalado
de datos existentes) para que el inventario se maneje siempre en las
unidades que usa la administradora. De paso, agrega un aviso tipo toast
en la esquina superior derecha al crear o editar recetas, subrecetas y
productos en el panel de analista, para que se note claramente si la
operacion tuvo exito o fallo sin tener que hacer scroll.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/plantilla_ingredientes.xlsx
+++ b/frontend/public/plantilla_ingredientes.xlsx
@@ -1,11 +1,19 @@
 
-<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Ingredientes" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>VARAGRILL — PLANTILLA DE CARGA DE INGREDIENTES</t>
   </si>
   <si>
-    <t>Completa Ingrediente, Unidad (kg, g, l, ml o unidad) y Cantidad. Deja la Cantidad vacía o en 0 en el ingrediente que NO quieras actualizar en esta carga — esa fila se ignora.</t>
+    <t>Completa Ingrediente, Unidad (g, ml o unidad) y Cantidad. Deja la Cantidad vacía o en 0 en el ingrediente que NO quieras actualizar en esta carga — esa fila se ignora.</t>
   </si>
   <si>
     <t>Ingrediente</t>
@@ -20,12 +28,12 @@
     <t>Tomate (ejemplo — reemplaza o borra esta fila)</t>
   </si>
   <si>
-    <t>kg</t>
+    <t>g</t>
   </si>
 </sst>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="4">
     <font>
@@ -88,15 +96,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Ingredientes" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
@@ -140,7 +140,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="0">
-        <v>20.5</v>
+        <v>20500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug de carga masiva soluccionado
</commit_message>
<xml_diff>
--- a/frontend/public/plantilla_ingredientes.xlsx
+++ b/frontend/public/plantilla_ingredientes.xlsx
@@ -8,12 +8,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>VARAGRILL — PLANTILLA DE CARGA DE INGREDIENTES</t>
   </si>
   <si>
-    <t>Completa Ingrediente, Unidad (g, ml o unidad) y Cantidad. Deja la Cantidad vacía o en 0 en el ingrediente que NO quieras actualizar en esta carga — esa fila se ignora.</t>
+    <t>Completa Ingrediente, Unidad (g, ml o unidad) y Cantidad. Deja la Cantidad vacía o en 0 en el ingrediente que NO quieras actualizar en esta carga — esa fila se ignora. Si además completas Peso neto, Peso real y Precio de compra (las tres juntas), el costo unitario se calcula solo; para un ingrediente que ya existe, esas tres columnas pueden ir solas, sin Cantidad, para actualizar el costeo sin hacer un reconteo.</t>
   </si>
   <si>
     <t>Ingrediente</t>
@@ -29,6 +29,15 @@
   </si>
   <si>
     <t>g</t>
+  </si>
+  <si>
+    <t>Peso neto</t>
+  </si>
+  <si>
+    <t>Peso real</t>
+  </si>
+  <si>
+    <t>Precio de compra</t>
   </si>
 </sst>
 </file>
@@ -98,30 +107,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="22" customHeight="1">
+    <row r="1" spans="1:6" ht="22" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:3" ht="30" customHeight="1">
+    <row r="2" spans="1:6" ht="45" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:3"/>
-    <row r="4" spans="1:3">
+    <row r="3" spans="1:6"/>
+    <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -131,8 +149,17 @@
       <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:6">
       <c r="A5" s="0" t="s">
         <v>5</v>
       </c>
@@ -142,11 +169,20 @@
       <c r="C5" s="0">
         <v>20500</v>
       </c>
+      <c r="D5" s="0">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="0">
+        <v>900</v>
+      </c>
+      <c r="F5" s="0">
+        <v>8500</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>